<commit_message>
[CBDDO & ZT-OT] Fix Framework Packager
</commit_message>
<xml_diff>
--- a/tools/excel/DoW/ZT-OT.xlsx
+++ b/tools/excel/DoW/ZT-OT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\DoW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FD544E-42DD-41A2-9042-43A9160BEFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4481DB63-03C7-4F48-B12C-7A556813D547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="907" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3645" yWindow="-14940" windowWidth="19665" windowHeight="14430" tabRatio="907" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -571,9 +571,6 @@
     <t>labels</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/celalunalp/</t>
-  </si>
-  <si>
     <t>USER</t>
   </si>
   <si>
@@ -2106,6 +2103,9 @@
   </si>
   <si>
     <t>urn:intuitem:risk:framework:zt_ot</t>
+  </si>
+  <si>
+    <t>celalunalp</t>
   </si>
 </sst>
 </file>
@@ -3548,7 +3548,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -3564,7 +3564,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -3572,7 +3572,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -3580,7 +3580,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
@@ -3588,7 +3588,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -3596,7 +3596,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -3604,7 +3604,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -3612,7 +3612,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>39</v>
+        <v>495</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3620,7 +3620,7 @@
         <v>38</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -3654,7 +3654,7 @@
         <v>13</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -3662,7 +3662,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -3670,7 +3670,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -3678,7 +3678,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
@@ -3686,7 +3686,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -3718,7 +3718,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="D2" s="37"/>
       <c r="E2" s="38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F2" s="39"/>
       <c r="G2" s="39"/>
@@ -3813,29 +3813,29 @@
         <v>2</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" s="43"/>
       <c r="E3" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="44" t="s">
+      <c r="G3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="43" t="s">
-        <v>44</v>
-      </c>
       <c r="H3" s="43" t="s">
         <v>37</v>
       </c>
       <c r="I3" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="45" t="s">
+      <c r="K3" s="55" t="s">
         <v>46</v>
-      </c>
-      <c r="K3" s="55" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="234.6" x14ac:dyDescent="0.3">
@@ -3846,29 +3846,29 @@
         <v>2</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D4" s="43"/>
       <c r="E4" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="44" t="s">
+      <c r="G4" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H4" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="46" t="s">
+      <c r="K4" s="55" t="s">
         <v>51</v>
-      </c>
-      <c r="K4" s="55" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -3879,29 +3879,29 @@
         <v>2</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" s="43"/>
       <c r="E5" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="44" t="s">
+      <c r="G5" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="46" t="s">
-        <v>56</v>
-      </c>
       <c r="K5" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -3912,29 +3912,29 @@
         <v>2</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6" s="43"/>
       <c r="E6" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="44" t="s">
+      <c r="G6" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="45" t="s">
+      <c r="K6" s="55" t="s">
         <v>60</v>
-      </c>
-      <c r="K6" s="55" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -3945,29 +3945,29 @@
         <v>2</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D7" s="43"/>
       <c r="E7" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="44" t="s">
+      <c r="G7" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="G7" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7" s="43" t="s">
+      <c r="J7" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="46" t="s">
+      <c r="K7" s="55" t="s">
         <v>66</v>
-      </c>
-      <c r="K7" s="55" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -3978,29 +3978,29 @@
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D8" s="43"/>
       <c r="E8" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="43" t="s">
+      <c r="G8" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J8" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I8" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J8" s="47" t="s">
-        <v>71</v>
-      </c>
       <c r="K8" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -4011,29 +4011,29 @@
         <v>2</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="43"/>
       <c r="E9" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="G9" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J9" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="G9" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H9" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J9" s="46" t="s">
-        <v>75</v>
-      </c>
       <c r="K9" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4044,29 +4044,29 @@
         <v>2</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D10" s="43"/>
       <c r="E10" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="G10" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="G10" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H10" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J10" s="46" t="s">
-        <v>79</v>
-      </c>
       <c r="K10" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -4077,29 +4077,29 @@
         <v>2</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="43"/>
       <c r="E11" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="G11" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I11" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J11" s="47" t="s">
         <v>82</v>
       </c>
-      <c r="G11" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H11" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I11" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J11" s="47" t="s">
-        <v>83</v>
-      </c>
       <c r="K11" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -4110,29 +4110,29 @@
         <v>2</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D12" s="43"/>
       <c r="E12" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="F12" s="44" t="s">
+      <c r="G12" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H12" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="G12" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I12" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J12" s="47" t="s">
-        <v>87</v>
-      </c>
       <c r="K12" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4143,29 +4143,29 @@
         <v>2</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="44" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="F13" s="44" t="s">
+      <c r="G13" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H13" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I13" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J13" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="G13" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H13" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I13" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J13" s="47" t="s">
-        <v>91</v>
-      </c>
       <c r="K13" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="151.80000000000001" x14ac:dyDescent="0.3">
@@ -4176,29 +4176,29 @@
         <v>2</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D14" s="43"/>
       <c r="E14" s="43" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="G14" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="G14" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H14" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I14" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J14" s="46" t="s">
-        <v>95</v>
-      </c>
       <c r="K14" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -4209,29 +4209,29 @@
         <v>2</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D15" s="43"/>
       <c r="E15" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="F15" s="44" t="s">
+      <c r="G15" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H15" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I15" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J15" s="47" t="s">
         <v>98</v>
       </c>
-      <c r="G15" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I15" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J15" s="47" t="s">
-        <v>99</v>
-      </c>
       <c r="K15" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -4242,29 +4242,29 @@
         <v>2</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D16" s="43"/>
       <c r="E16" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="44" t="s">
         <v>101</v>
       </c>
-      <c r="F16" s="44" t="s">
+      <c r="G16" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J16" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="G16" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H16" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I16" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J16" s="46" t="s">
-        <v>103</v>
-      </c>
       <c r="K16" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="55.2" x14ac:dyDescent="0.3">
@@ -4275,29 +4275,29 @@
         <v>2</v>
       </c>
       <c r="C17" s="43" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D17" s="43"/>
       <c r="E17" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="44" t="s">
+      <c r="G17" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I17" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J17" s="47" t="s">
         <v>106</v>
       </c>
-      <c r="G17" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H17" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I17" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J17" s="47" t="s">
-        <v>107</v>
-      </c>
       <c r="K17" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="179.4" x14ac:dyDescent="0.3">
@@ -4308,29 +4308,29 @@
         <v>2</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D18" s="43"/>
       <c r="E18" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="44" t="s">
         <v>109</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="G18" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" s="46" t="s">
         <v>110</v>
       </c>
-      <c r="G18" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H18" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I18" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J18" s="46" t="s">
-        <v>111</v>
-      </c>
       <c r="K18" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="179.4" x14ac:dyDescent="0.3">
@@ -4341,29 +4341,29 @@
         <v>2</v>
       </c>
       <c r="C19" s="43" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D19" s="43"/>
       <c r="E19" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="F19" s="44" t="s">
+      <c r="G19" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I19" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J19" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="G19" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H19" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I19" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J19" s="48" t="s">
-        <v>115</v>
-      </c>
       <c r="K19" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -4374,29 +4374,29 @@
         <v>2</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D20" s="43"/>
       <c r="E20" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="43" t="s">
         <v>117</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="G20" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="H20" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I20" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J20" s="45" t="s">
         <v>118</v>
       </c>
-      <c r="G20" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I20" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J20" s="45" t="s">
-        <v>119</v>
-      </c>
       <c r="K20" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="D21" s="43"/>
       <c r="E21" s="44" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F21" s="43"/>
       <c r="G21" s="43"/>
@@ -4426,29 +4426,29 @@
         <v>2</v>
       </c>
       <c r="C22" s="43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D22" s="43"/>
       <c r="E22" s="43" t="s">
+        <v>121</v>
+      </c>
+      <c r="F22" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="G22" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="G22" s="43" t="s">
+      <c r="H22" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I22" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J22" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="H22" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I22" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J22" s="49" t="s">
-        <v>125</v>
-      </c>
       <c r="K22" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="179.4" x14ac:dyDescent="0.3">
@@ -4459,29 +4459,29 @@
         <v>2</v>
       </c>
       <c r="C23" s="43" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D23" s="43"/>
       <c r="E23" s="43" t="s">
+        <v>126</v>
+      </c>
+      <c r="F23" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="G23" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I23" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J23" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="G23" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H23" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I23" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J23" s="49" t="s">
-        <v>129</v>
-      </c>
       <c r="K23" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="187.2" x14ac:dyDescent="0.3">
@@ -4492,29 +4492,29 @@
         <v>2</v>
       </c>
       <c r="C24" s="43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D24" s="43"/>
       <c r="E24" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="F24" s="44" t="s">
+      <c r="G24" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I24" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J24" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="G24" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H24" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I24" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J24" s="49" t="s">
+      <c r="K24" s="55" t="s">
         <v>133</v>
-      </c>
-      <c r="K24" s="55" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="151.80000000000001" x14ac:dyDescent="0.3">
@@ -4525,29 +4525,29 @@
         <v>2</v>
       </c>
       <c r="C25" s="43" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D25" s="43"/>
       <c r="E25" s="43" t="s">
+        <v>135</v>
+      </c>
+      <c r="F25" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="F25" s="44" t="s">
+      <c r="G25" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I25" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J25" s="46" t="s">
         <v>137</v>
       </c>
-      <c r="G25" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H25" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I25" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" s="46" t="s">
-        <v>138</v>
-      </c>
       <c r="K25" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="187.2" x14ac:dyDescent="0.3">
@@ -4558,29 +4558,29 @@
         <v>2</v>
       </c>
       <c r="C26" s="43" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D26" s="43"/>
       <c r="E26" s="43" t="s">
+        <v>139</v>
+      </c>
+      <c r="F26" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="F26" s="43" t="s">
+      <c r="G26" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H26" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I26" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J26" s="49" t="s">
         <v>141</v>
       </c>
-      <c r="G26" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H26" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I26" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J26" s="49" t="s">
-        <v>142</v>
-      </c>
       <c r="K26" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4591,29 +4591,29 @@
         <v>2</v>
       </c>
       <c r="C27" s="43" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D27" s="43"/>
       <c r="E27" s="43" t="s">
+        <v>143</v>
+      </c>
+      <c r="F27" s="44" t="s">
         <v>144</v>
       </c>
-      <c r="F27" s="44" t="s">
+      <c r="G27" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H27" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I27" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J27" s="49" t="s">
         <v>145</v>
       </c>
-      <c r="G27" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H27" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I27" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J27" s="49" t="s">
-        <v>146</v>
-      </c>
       <c r="K27" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -4624,29 +4624,29 @@
         <v>2</v>
       </c>
       <c r="C28" s="43" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D28" s="43"/>
       <c r="E28" s="43" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" s="44" t="s">
         <v>148</v>
       </c>
-      <c r="F28" s="44" t="s">
+      <c r="G28" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H28" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I28" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J28" s="49" t="s">
         <v>149</v>
       </c>
-      <c r="G28" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H28" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I28" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J28" s="49" t="s">
-        <v>150</v>
-      </c>
       <c r="K28" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -4657,29 +4657,29 @@
         <v>2</v>
       </c>
       <c r="C29" s="43" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D29" s="43"/>
       <c r="E29" s="43" t="s">
+        <v>151</v>
+      </c>
+      <c r="F29" s="43" t="s">
         <v>152</v>
       </c>
-      <c r="F29" s="43" t="s">
+      <c r="G29" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H29" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I29" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J29" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="G29" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H29" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I29" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J29" s="46" t="s">
-        <v>154</v>
-      </c>
       <c r="K29" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -4690,29 +4690,29 @@
         <v>2</v>
       </c>
       <c r="C30" s="43" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D30" s="43"/>
       <c r="E30" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="F30" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="F30" s="44" t="s">
+      <c r="G30" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H30" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I30" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J30" s="49" t="s">
         <v>157</v>
       </c>
-      <c r="G30" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H30" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I30" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J30" s="49" t="s">
-        <v>158</v>
-      </c>
       <c r="K30" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -4723,29 +4723,29 @@
         <v>2</v>
       </c>
       <c r="C31" s="43" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D31" s="43"/>
       <c r="E31" s="43" t="s">
+        <v>159</v>
+      </c>
+      <c r="F31" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="F31" s="44" t="s">
+      <c r="G31" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H31" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I31" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J31" s="45" t="s">
         <v>161</v>
       </c>
-      <c r="G31" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H31" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I31" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J31" s="45" t="s">
-        <v>162</v>
-      </c>
       <c r="K31" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -4756,29 +4756,29 @@
         <v>2</v>
       </c>
       <c r="C32" s="43" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D32" s="43"/>
       <c r="E32" s="43" t="s">
+        <v>163</v>
+      </c>
+      <c r="F32" s="43" t="s">
         <v>164</v>
       </c>
-      <c r="F32" s="43" t="s">
+      <c r="G32" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H32" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I32" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J32" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="G32" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H32" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I32" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J32" s="47" t="s">
-        <v>166</v>
-      </c>
       <c r="K32" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="179.4" x14ac:dyDescent="0.3">
@@ -4789,29 +4789,29 @@
         <v>2</v>
       </c>
       <c r="C33" s="43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D33" s="43"/>
       <c r="E33" s="43" t="s">
+        <v>167</v>
+      </c>
+      <c r="F33" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="F33" s="44" t="s">
+      <c r="G33" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H33" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I33" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J33" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="G33" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H33" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I33" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J33" s="46" t="s">
-        <v>170</v>
-      </c>
       <c r="K33" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="55.2" x14ac:dyDescent="0.3">
@@ -4822,29 +4822,29 @@
         <v>2</v>
       </c>
       <c r="C34" s="43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D34" s="43"/>
       <c r="E34" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="F34" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="F34" s="44" t="s">
+      <c r="G34" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H34" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I34" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J34" s="45" t="s">
         <v>173</v>
       </c>
-      <c r="G34" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H34" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I34" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J34" s="45" t="s">
-        <v>174</v>
-      </c>
       <c r="K34" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4855,29 +4855,29 @@
         <v>2</v>
       </c>
       <c r="C35" s="43" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D35" s="43"/>
       <c r="E35" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="F35" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="F35" s="44" t="s">
+      <c r="G35" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H35" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I35" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J35" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="G35" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H35" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I35" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J35" s="50" t="s">
-        <v>178</v>
-      </c>
       <c r="K35" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4888,29 +4888,29 @@
         <v>2</v>
       </c>
       <c r="C36" s="43" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D36" s="43"/>
       <c r="E36" s="44" t="s">
+        <v>179</v>
+      </c>
+      <c r="F36" s="44" t="s">
         <v>180</v>
       </c>
-      <c r="F36" s="44" t="s">
+      <c r="G36" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H36" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I36" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J36" s="44" t="s">
         <v>181</v>
       </c>
-      <c r="G36" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H36" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I36" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J36" s="44" t="s">
-        <v>182</v>
-      </c>
       <c r="K36" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -4921,29 +4921,29 @@
         <v>2</v>
       </c>
       <c r="C37" s="43" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D37" s="43"/>
       <c r="E37" s="43" t="s">
+        <v>183</v>
+      </c>
+      <c r="F37" s="44" t="s">
         <v>184</v>
       </c>
-      <c r="F37" s="44" t="s">
+      <c r="G37" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="H37" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I37" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J37" s="51" t="s">
         <v>185</v>
       </c>
-      <c r="G37" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="H37" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I37" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J37" s="51" t="s">
-        <v>186</v>
-      </c>
       <c r="K37" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D38" s="43"/>
       <c r="E38" s="43" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F38" s="44"/>
       <c r="G38" s="43"/>
@@ -4973,29 +4973,29 @@
         <v>2</v>
       </c>
       <c r="C39" s="43" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D39" s="43"/>
       <c r="E39" s="43" t="s">
+        <v>188</v>
+      </c>
+      <c r="F39" s="44" t="s">
         <v>189</v>
       </c>
-      <c r="F39" s="44" t="s">
+      <c r="G39" s="43" t="s">
         <v>190</v>
       </c>
-      <c r="G39" s="43" t="s">
+      <c r="H39" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I39" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J39" s="44" t="s">
         <v>191</v>
       </c>
-      <c r="H39" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I39" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J39" s="44" t="s">
-        <v>192</v>
-      </c>
       <c r="K39" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="55.2" x14ac:dyDescent="0.3">
@@ -5006,29 +5006,29 @@
         <v>2</v>
       </c>
       <c r="C40" s="43" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D40" s="43"/>
       <c r="E40" s="52" t="s">
+        <v>193</v>
+      </c>
+      <c r="F40" s="44" t="s">
         <v>194</v>
       </c>
-      <c r="F40" s="44" t="s">
+      <c r="G40" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="H40" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I40" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J40" s="44" t="s">
         <v>195</v>
       </c>
-      <c r="G40" s="44" t="s">
-        <v>191</v>
-      </c>
-      <c r="H40" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I40" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J40" s="44" t="s">
-        <v>196</v>
-      </c>
       <c r="K40" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -5039,29 +5039,29 @@
         <v>2</v>
       </c>
       <c r="C41" s="43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D41" s="43"/>
       <c r="E41" s="43" t="s">
+        <v>197</v>
+      </c>
+      <c r="F41" s="44" t="s">
         <v>198</v>
       </c>
-      <c r="F41" s="44" t="s">
+      <c r="G41" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H41" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I41" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J41" s="44" t="s">
         <v>199</v>
       </c>
-      <c r="G41" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H41" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I41" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J41" s="44" t="s">
-        <v>200</v>
-      </c>
       <c r="K41" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -5072,29 +5072,29 @@
         <v>2</v>
       </c>
       <c r="C42" s="43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D42" s="43"/>
       <c r="E42" s="43" t="s">
+        <v>201</v>
+      </c>
+      <c r="F42" s="51" t="s">
         <v>202</v>
       </c>
-      <c r="F42" s="51" t="s">
+      <c r="G42" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H42" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I42" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J42" s="43" t="s">
         <v>203</v>
       </c>
-      <c r="G42" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H42" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I42" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J42" s="43" t="s">
-        <v>204</v>
-      </c>
       <c r="K42" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -5105,29 +5105,29 @@
         <v>2</v>
       </c>
       <c r="C43" s="43" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D43" s="43"/>
       <c r="E43" s="43" t="s">
+        <v>205</v>
+      </c>
+      <c r="F43" s="43" t="s">
         <v>206</v>
       </c>
-      <c r="F43" s="43" t="s">
+      <c r="G43" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H43" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I43" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J43" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="G43" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H43" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I43" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J43" s="51" t="s">
-        <v>208</v>
-      </c>
       <c r="K43" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -5138,29 +5138,29 @@
         <v>2</v>
       </c>
       <c r="C44" s="43" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D44" s="43"/>
       <c r="E44" s="43" t="s">
+        <v>209</v>
+      </c>
+      <c r="F44" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="F44" s="44" t="s">
+      <c r="G44" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H44" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I44" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J44" s="50" t="s">
         <v>211</v>
       </c>
-      <c r="G44" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H44" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I44" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J44" s="50" t="s">
-        <v>212</v>
-      </c>
       <c r="K44" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -5171,29 +5171,29 @@
         <v>2</v>
       </c>
       <c r="C45" s="43" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D45" s="43"/>
       <c r="E45" s="43" t="s">
+        <v>213</v>
+      </c>
+      <c r="F45" s="44" t="s">
         <v>214</v>
       </c>
-      <c r="F45" s="44" t="s">
+      <c r="G45" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H45" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I45" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J45" s="50" t="s">
         <v>215</v>
       </c>
-      <c r="G45" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H45" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I45" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J45" s="50" t="s">
-        <v>216</v>
-      </c>
       <c r="K45" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -5204,29 +5204,29 @@
         <v>2</v>
       </c>
       <c r="C46" s="43" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D46" s="43"/>
       <c r="E46" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="F46" s="44" t="s">
         <v>218</v>
       </c>
-      <c r="F46" s="44" t="s">
+      <c r="G46" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H46" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I46" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J46" s="43" t="s">
         <v>219</v>
       </c>
-      <c r="G46" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H46" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I46" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J46" s="43" t="s">
-        <v>220</v>
-      </c>
       <c r="K46" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
@@ -5237,29 +5237,29 @@
         <v>2</v>
       </c>
       <c r="C47" s="43" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D47" s="43"/>
       <c r="E47" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="F47" s="44" t="s">
         <v>222</v>
       </c>
-      <c r="F47" s="44" t="s">
+      <c r="G47" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H47" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I47" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J47" s="50" t="s">
         <v>223</v>
       </c>
-      <c r="G47" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H47" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I47" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J47" s="50" t="s">
-        <v>224</v>
-      </c>
       <c r="K47" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
@@ -5270,29 +5270,29 @@
         <v>2</v>
       </c>
       <c r="C48" s="43" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D48" s="43"/>
       <c r="E48" s="43" t="s">
+        <v>225</v>
+      </c>
+      <c r="F48" s="44" t="s">
         <v>226</v>
       </c>
-      <c r="F48" s="44" t="s">
+      <c r="G48" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="H48" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I48" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J48" s="50" t="s">
         <v>227</v>
       </c>
-      <c r="G48" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="H48" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I48" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J48" s="50" t="s">
-        <v>228</v>
-      </c>
       <c r="K48" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -5303,29 +5303,29 @@
         <v>2</v>
       </c>
       <c r="C49" s="43" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D49" s="43"/>
       <c r="E49" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="F49" s="44" t="s">
         <v>230</v>
       </c>
-      <c r="F49" s="44" t="s">
+      <c r="G49" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="H49" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I49" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J49" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="G49" s="44" t="s">
-        <v>191</v>
-      </c>
-      <c r="H49" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I49" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J49" s="44" t="s">
-        <v>232</v>
-      </c>
       <c r="K49" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -5336,29 +5336,29 @@
         <v>2</v>
       </c>
       <c r="C50" s="43" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D50" s="43"/>
       <c r="E50" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="F50" s="52" t="s">
         <v>234</v>
       </c>
-      <c r="F50" s="52" t="s">
+      <c r="G50" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="H50" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I50" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J50" s="44" t="s">
         <v>235</v>
       </c>
-      <c r="G50" s="44" t="s">
-        <v>191</v>
-      </c>
-      <c r="H50" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I50" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J50" s="44" t="s">
-        <v>236</v>
-      </c>
       <c r="K50" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="D51" s="43"/>
       <c r="E51" s="44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F51" s="52"/>
       <c r="G51" s="44"/>
@@ -5388,29 +5388,29 @@
         <v>2</v>
       </c>
       <c r="C52" s="43" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D52" s="43"/>
       <c r="E52" s="43" t="s">
+        <v>238</v>
+      </c>
+      <c r="F52" s="43" t="s">
         <v>239</v>
       </c>
-      <c r="F52" s="43" t="s">
+      <c r="G52" s="43" t="s">
         <v>240</v>
       </c>
-      <c r="G52" s="43" t="s">
+      <c r="H52" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I52" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J52" s="50" t="s">
         <v>241</v>
       </c>
-      <c r="H52" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I52" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J52" s="50" t="s">
-        <v>242</v>
-      </c>
       <c r="K52" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="151.80000000000001" x14ac:dyDescent="0.3">
@@ -5421,29 +5421,29 @@
         <v>2</v>
       </c>
       <c r="C53" s="43" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D53" s="43"/>
       <c r="E53" s="43" t="s">
+        <v>243</v>
+      </c>
+      <c r="F53" s="44" t="s">
         <v>244</v>
       </c>
-      <c r="F53" s="44" t="s">
+      <c r="G53" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H53" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I53" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J53" s="50" t="s">
         <v>245</v>
       </c>
-      <c r="G53" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H53" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I53" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J53" s="50" t="s">
-        <v>246</v>
-      </c>
       <c r="K53" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -5454,29 +5454,29 @@
         <v>2</v>
       </c>
       <c r="C54" s="43" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D54" s="43"/>
       <c r="E54" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="F54" s="44" t="s">
         <v>248</v>
       </c>
-      <c r="F54" s="44" t="s">
+      <c r="G54" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H54" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I54" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J54" s="50" t="s">
         <v>249</v>
       </c>
-      <c r="G54" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H54" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I54" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J54" s="50" t="s">
-        <v>250</v>
-      </c>
       <c r="K54" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="244.8" x14ac:dyDescent="0.3">
@@ -5487,29 +5487,29 @@
         <v>2</v>
       </c>
       <c r="C55" s="43" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D55" s="43"/>
       <c r="E55" s="43" t="s">
+        <v>251</v>
+      </c>
+      <c r="F55" s="43" t="s">
         <v>252</v>
       </c>
-      <c r="F55" s="43" t="s">
+      <c r="G55" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H55" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I55" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J55" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="G55" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H55" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I55" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J55" s="50" t="s">
-        <v>254</v>
-      </c>
       <c r="K55" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -5520,29 +5520,29 @@
         <v>2</v>
       </c>
       <c r="C56" s="43" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D56" s="43"/>
       <c r="E56" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="F56" s="44" t="s">
         <v>256</v>
       </c>
-      <c r="F56" s="44" t="s">
+      <c r="G56" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H56" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I56" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J56" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="G56" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H56" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I56" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J56" s="50" t="s">
-        <v>258</v>
-      </c>
       <c r="K56" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -5553,29 +5553,29 @@
         <v>2</v>
       </c>
       <c r="C57" s="43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D57" s="43"/>
       <c r="E57" s="43" t="s">
+        <v>259</v>
+      </c>
+      <c r="F57" s="44" t="s">
         <v>260</v>
       </c>
-      <c r="F57" s="44" t="s">
+      <c r="G57" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H57" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I57" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J57" s="43" t="s">
         <v>261</v>
       </c>
-      <c r="G57" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H57" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I57" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J57" s="43" t="s">
-        <v>262</v>
-      </c>
       <c r="K57" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -5586,29 +5586,29 @@
         <v>2</v>
       </c>
       <c r="C58" s="43" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D58" s="43"/>
       <c r="E58" s="43" t="s">
+        <v>263</v>
+      </c>
+      <c r="F58" s="44" t="s">
         <v>264</v>
       </c>
-      <c r="F58" s="44" t="s">
+      <c r="G58" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H58" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I58" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J58" s="51" t="s">
         <v>265</v>
       </c>
-      <c r="G58" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H58" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I58" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J58" s="51" t="s">
-        <v>266</v>
-      </c>
       <c r="K58" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -5619,29 +5619,29 @@
         <v>2</v>
       </c>
       <c r="C59" s="43" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D59" s="43"/>
       <c r="E59" s="43" t="s">
+        <v>267</v>
+      </c>
+      <c r="F59" s="44" t="s">
         <v>268</v>
       </c>
-      <c r="F59" s="44" t="s">
+      <c r="G59" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H59" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I59" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J59" s="50" t="s">
         <v>269</v>
       </c>
-      <c r="G59" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H59" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I59" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J59" s="50" t="s">
-        <v>270</v>
-      </c>
       <c r="K59" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -5652,29 +5652,29 @@
         <v>2</v>
       </c>
       <c r="C60" s="43" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D60" s="43"/>
       <c r="E60" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="F60" s="44" t="s">
         <v>272</v>
       </c>
-      <c r="F60" s="44" t="s">
+      <c r="G60" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H60" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I60" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J60" s="51" t="s">
         <v>273</v>
       </c>
-      <c r="G60" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H60" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I60" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J60" s="51" t="s">
-        <v>274</v>
-      </c>
       <c r="K60" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="55.2" x14ac:dyDescent="0.3">
@@ -5685,29 +5685,29 @@
         <v>2</v>
       </c>
       <c r="C61" s="43" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D61" s="43"/>
       <c r="E61" s="43" t="s">
+        <v>275</v>
+      </c>
+      <c r="F61" s="43" t="s">
         <v>276</v>
       </c>
-      <c r="F61" s="43" t="s">
+      <c r="G61" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H61" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I61" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J61" s="51" t="s">
         <v>277</v>
       </c>
-      <c r="G61" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H61" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I61" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J61" s="51" t="s">
-        <v>278</v>
-      </c>
       <c r="K61" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -5718,29 +5718,29 @@
         <v>2</v>
       </c>
       <c r="C62" s="43" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D62" s="43"/>
       <c r="E62" s="43" t="s">
+        <v>279</v>
+      </c>
+      <c r="F62" s="43" t="s">
         <v>280</v>
       </c>
-      <c r="F62" s="43" t="s">
+      <c r="G62" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H62" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I62" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J62" s="43" t="s">
         <v>281</v>
       </c>
-      <c r="G62" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H62" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I62" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J62" s="43" t="s">
-        <v>282</v>
-      </c>
       <c r="K62" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="144" x14ac:dyDescent="0.3">
@@ -5751,29 +5751,29 @@
         <v>2</v>
       </c>
       <c r="C63" s="43" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D63" s="43"/>
       <c r="E63" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="F63" s="44" t="s">
         <v>284</v>
       </c>
-      <c r="F63" s="44" t="s">
+      <c r="G63" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H63" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I63" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J63" s="50" t="s">
         <v>285</v>
       </c>
-      <c r="G63" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H63" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I63" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J63" s="50" t="s">
-        <v>286</v>
-      </c>
       <c r="K63" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -5784,29 +5784,29 @@
         <v>2</v>
       </c>
       <c r="C64" s="43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D64" s="43"/>
       <c r="E64" s="43" t="s">
+        <v>287</v>
+      </c>
+      <c r="F64" s="44" t="s">
         <v>288</v>
       </c>
-      <c r="F64" s="44" t="s">
+      <c r="G64" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H64" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I64" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J64" s="43" t="s">
         <v>289</v>
       </c>
-      <c r="G64" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H64" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I64" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J64" s="43" t="s">
-        <v>290</v>
-      </c>
       <c r="K64" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
@@ -5817,29 +5817,29 @@
         <v>2</v>
       </c>
       <c r="C65" s="43" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D65" s="43"/>
       <c r="E65" s="43" t="s">
+        <v>291</v>
+      </c>
+      <c r="F65" s="44" t="s">
         <v>292</v>
       </c>
-      <c r="F65" s="44" t="s">
+      <c r="G65" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H65" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I65" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J65" s="50" t="s">
         <v>293</v>
       </c>
-      <c r="G65" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H65" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I65" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J65" s="50" t="s">
-        <v>294</v>
-      </c>
       <c r="K65" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
@@ -5850,29 +5850,29 @@
         <v>2</v>
       </c>
       <c r="C66" s="43" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D66" s="43"/>
       <c r="E66" s="43" t="s">
+        <v>295</v>
+      </c>
+      <c r="F66" s="43" t="s">
         <v>296</v>
       </c>
-      <c r="F66" s="43" t="s">
+      <c r="G66" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H66" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I66" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J66" s="50" t="s">
         <v>297</v>
       </c>
-      <c r="G66" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H66" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I66" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J66" s="50" t="s">
-        <v>298</v>
-      </c>
       <c r="K66" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -5883,29 +5883,29 @@
         <v>2</v>
       </c>
       <c r="C67" s="43" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D67" s="43"/>
       <c r="E67" s="43" t="s">
+        <v>299</v>
+      </c>
+      <c r="F67" s="44" t="s">
         <v>300</v>
       </c>
-      <c r="F67" s="44" t="s">
+      <c r="G67" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H67" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I67" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J67" s="50" t="s">
         <v>301</v>
       </c>
-      <c r="G67" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H67" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I67" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J67" s="50" t="s">
-        <v>302</v>
-      </c>
       <c r="K67" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
@@ -5916,29 +5916,29 @@
         <v>2</v>
       </c>
       <c r="C68" s="43" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D68" s="43"/>
       <c r="E68" s="43" t="s">
+        <v>303</v>
+      </c>
+      <c r="F68" s="43" t="s">
         <v>304</v>
       </c>
-      <c r="F68" s="43" t="s">
+      <c r="G68" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H68" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I68" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J68" s="50" t="s">
         <v>305</v>
       </c>
-      <c r="G68" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H68" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I68" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J68" s="50" t="s">
-        <v>306</v>
-      </c>
       <c r="K68" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -5949,29 +5949,29 @@
         <v>2</v>
       </c>
       <c r="C69" s="43" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D69" s="43"/>
       <c r="E69" s="43" t="s">
+        <v>307</v>
+      </c>
+      <c r="F69" s="44" t="s">
         <v>308</v>
       </c>
-      <c r="F69" s="44" t="s">
+      <c r="G69" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H69" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I69" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J69" s="51" t="s">
         <v>309</v>
       </c>
-      <c r="G69" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H69" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I69" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J69" s="51" t="s">
-        <v>310</v>
-      </c>
       <c r="K69" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -5982,29 +5982,29 @@
         <v>2</v>
       </c>
       <c r="C70" s="43" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D70" s="43"/>
       <c r="E70" s="43" t="s">
+        <v>311</v>
+      </c>
+      <c r="F70" s="43" t="s">
         <v>312</v>
       </c>
-      <c r="F70" s="43" t="s">
+      <c r="G70" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="H70" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I70" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J70" s="43" t="s">
         <v>313</v>
       </c>
-      <c r="G70" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H70" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I70" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J70" s="43" t="s">
-        <v>314</v>
-      </c>
       <c r="K70" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="D71" s="43"/>
       <c r="E71" s="43" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F71" s="43"/>
       <c r="G71" s="43"/>
@@ -6034,29 +6034,29 @@
         <v>2</v>
       </c>
       <c r="C72" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D72" s="43"/>
       <c r="E72" s="43" t="s">
+        <v>316</v>
+      </c>
+      <c r="F72" s="44" t="s">
         <v>317</v>
       </c>
-      <c r="F72" s="44" t="s">
+      <c r="G72" s="43" t="s">
         <v>318</v>
       </c>
-      <c r="G72" s="43" t="s">
+      <c r="H72" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I72" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J72" s="51" t="s">
         <v>319</v>
       </c>
-      <c r="H72" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I72" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J72" s="51" t="s">
-        <v>320</v>
-      </c>
       <c r="K72" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
@@ -6067,29 +6067,29 @@
         <v>2</v>
       </c>
       <c r="C73" s="43" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D73" s="43"/>
       <c r="E73" s="43" t="s">
+        <v>321</v>
+      </c>
+      <c r="F73" s="43" t="s">
         <v>322</v>
       </c>
-      <c r="F73" s="43" t="s">
+      <c r="G73" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H73" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I73" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J73" s="50" t="s">
         <v>323</v>
       </c>
-      <c r="G73" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H73" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I73" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J73" s="50" t="s">
-        <v>324</v>
-      </c>
       <c r="K73" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -6100,29 +6100,29 @@
         <v>2</v>
       </c>
       <c r="C74" s="43" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D74" s="43"/>
       <c r="E74" s="44" t="s">
+        <v>325</v>
+      </c>
+      <c r="F74" s="44" t="s">
         <v>326</v>
       </c>
-      <c r="F74" s="44" t="s">
+      <c r="G74" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H74" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I74" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J74" s="44" t="s">
         <v>327</v>
       </c>
-      <c r="G74" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H74" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I74" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J74" s="44" t="s">
-        <v>328</v>
-      </c>
       <c r="K74" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -6133,29 +6133,29 @@
         <v>2</v>
       </c>
       <c r="C75" s="43" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D75" s="43"/>
       <c r="E75" s="43" t="s">
+        <v>329</v>
+      </c>
+      <c r="F75" s="44" t="s">
         <v>330</v>
       </c>
-      <c r="F75" s="44" t="s">
+      <c r="G75" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H75" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I75" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J75" s="51" t="s">
         <v>331</v>
       </c>
-      <c r="G75" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H75" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I75" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J75" s="51" t="s">
-        <v>332</v>
-      </c>
       <c r="K75" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -6166,29 +6166,29 @@
         <v>2</v>
       </c>
       <c r="C76" s="43" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D76" s="43"/>
       <c r="E76" s="44" t="s">
+        <v>333</v>
+      </c>
+      <c r="F76" s="44" t="s">
         <v>334</v>
       </c>
-      <c r="F76" s="44" t="s">
+      <c r="G76" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H76" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I76" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J76" s="50" t="s">
         <v>335</v>
       </c>
-      <c r="G76" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H76" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I76" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J76" s="50" t="s">
-        <v>336</v>
-      </c>
       <c r="K76" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6199,29 +6199,29 @@
         <v>2</v>
       </c>
       <c r="C77" s="43" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D77" s="43"/>
       <c r="E77" s="43" t="s">
+        <v>337</v>
+      </c>
+      <c r="F77" s="44" t="s">
         <v>338</v>
       </c>
-      <c r="F77" s="44" t="s">
+      <c r="G77" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H77" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I77" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J77" s="50" t="s">
         <v>339</v>
       </c>
-      <c r="G77" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H77" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I77" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J77" s="50" t="s">
-        <v>340</v>
-      </c>
       <c r="K77" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
@@ -6232,29 +6232,29 @@
         <v>2</v>
       </c>
       <c r="C78" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D78" s="43"/>
       <c r="E78" s="52" t="s">
+        <v>341</v>
+      </c>
+      <c r="F78" s="44" t="s">
         <v>342</v>
       </c>
-      <c r="F78" s="44" t="s">
+      <c r="G78" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H78" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I78" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J78" s="50" t="s">
         <v>343</v>
       </c>
-      <c r="G78" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H78" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I78" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J78" s="50" t="s">
-        <v>344</v>
-      </c>
       <c r="K78" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="151.80000000000001" x14ac:dyDescent="0.3">
@@ -6265,29 +6265,29 @@
         <v>2</v>
       </c>
       <c r="C79" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D79" s="43"/>
       <c r="E79" s="43" t="s">
+        <v>345</v>
+      </c>
+      <c r="F79" s="44" t="s">
         <v>346</v>
       </c>
-      <c r="F79" s="44" t="s">
+      <c r="G79" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H79" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I79" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J79" s="50" t="s">
         <v>347</v>
       </c>
-      <c r="G79" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H79" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I79" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J79" s="50" t="s">
-        <v>348</v>
-      </c>
       <c r="K79" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -6298,29 +6298,29 @@
         <v>2</v>
       </c>
       <c r="C80" s="43" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D80" s="43"/>
       <c r="E80" s="43" t="s">
+        <v>349</v>
+      </c>
+      <c r="F80" s="44" t="s">
         <v>350</v>
       </c>
-      <c r="F80" s="44" t="s">
+      <c r="G80" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H80" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I80" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J80" s="44" t="s">
         <v>351</v>
       </c>
-      <c r="G80" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H80" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I80" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J80" s="44" t="s">
-        <v>352</v>
-      </c>
       <c r="K80" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -6331,29 +6331,29 @@
         <v>2</v>
       </c>
       <c r="C81" s="43" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D81" s="43"/>
       <c r="E81" s="44" t="s">
+        <v>353</v>
+      </c>
+      <c r="F81" s="44" t="s">
         <v>354</v>
       </c>
-      <c r="F81" s="44" t="s">
+      <c r="G81" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="H81" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I81" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J81" s="44" t="s">
         <v>355</v>
       </c>
-      <c r="G81" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="H81" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I81" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J81" s="44" t="s">
-        <v>356</v>
-      </c>
       <c r="K81" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="D82" s="43"/>
       <c r="E82" s="44" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F82" s="44"/>
       <c r="G82" s="43"/>
@@ -6383,29 +6383,29 @@
         <v>2</v>
       </c>
       <c r="C83" s="43" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D83" s="43"/>
       <c r="E83" s="43" t="s">
+        <v>358</v>
+      </c>
+      <c r="F83" s="44" t="s">
         <v>359</v>
       </c>
-      <c r="F83" s="44" t="s">
+      <c r="G83" s="43" t="s">
         <v>360</v>
       </c>
-      <c r="G83" s="43" t="s">
+      <c r="H83" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I83" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J83" s="50" t="s">
         <v>361</v>
       </c>
-      <c r="H83" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I83" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J83" s="50" t="s">
-        <v>362</v>
-      </c>
       <c r="K83" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -6416,29 +6416,29 @@
         <v>2</v>
       </c>
       <c r="C84" s="43" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D84" s="43"/>
       <c r="E84" s="43" t="s">
+        <v>363</v>
+      </c>
+      <c r="F84" s="44" t="s">
         <v>364</v>
       </c>
-      <c r="F84" s="44" t="s">
+      <c r="G84" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H84" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I84" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J84" s="50" t="s">
         <v>365</v>
       </c>
-      <c r="G84" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H84" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I84" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J84" s="50" t="s">
-        <v>366</v>
-      </c>
       <c r="K84" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
@@ -6449,29 +6449,29 @@
         <v>2</v>
       </c>
       <c r="C85" s="43" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D85" s="43"/>
       <c r="E85" s="44" t="s">
+        <v>367</v>
+      </c>
+      <c r="F85" s="44" t="s">
         <v>368</v>
       </c>
-      <c r="F85" s="44" t="s">
+      <c r="G85" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H85" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I85" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J85" s="50" t="s">
         <v>369</v>
       </c>
-      <c r="G85" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H85" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I85" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J85" s="50" t="s">
-        <v>370</v>
-      </c>
       <c r="K85" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -6482,29 +6482,29 @@
         <v>2</v>
       </c>
       <c r="C86" s="43" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D86" s="43"/>
       <c r="E86" s="44" t="s">
+        <v>371</v>
+      </c>
+      <c r="F86" s="43" t="s">
         <v>372</v>
       </c>
-      <c r="F86" s="43" t="s">
+      <c r="G86" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H86" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I86" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J86" s="43" t="s">
         <v>373</v>
       </c>
-      <c r="G86" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H86" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I86" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J86" s="43" t="s">
-        <v>374</v>
-      </c>
       <c r="K86" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
@@ -6515,29 +6515,29 @@
         <v>2</v>
       </c>
       <c r="C87" s="43" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D87" s="43"/>
       <c r="E87" s="44" t="s">
+        <v>375</v>
+      </c>
+      <c r="F87" s="44" t="s">
         <v>376</v>
       </c>
-      <c r="F87" s="44" t="s">
+      <c r="G87" s="44" t="s">
+        <v>360</v>
+      </c>
+      <c r="H87" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I87" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J87" s="50" t="s">
         <v>377</v>
       </c>
-      <c r="G87" s="44" t="s">
-        <v>361</v>
-      </c>
-      <c r="H87" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I87" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J87" s="50" t="s">
-        <v>378</v>
-      </c>
       <c r="K87" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6548,29 +6548,29 @@
         <v>2</v>
       </c>
       <c r="C88" s="43" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D88" s="43"/>
       <c r="E88" s="43" t="s">
+        <v>379</v>
+      </c>
+      <c r="F88" s="43" t="s">
         <v>380</v>
       </c>
-      <c r="F88" s="43" t="s">
+      <c r="G88" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H88" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I88" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J88" s="51" t="s">
         <v>381</v>
       </c>
-      <c r="G88" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H88" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I88" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J88" s="51" t="s">
-        <v>382</v>
-      </c>
       <c r="K88" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6581,29 +6581,29 @@
         <v>2</v>
       </c>
       <c r="C89" s="43" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D89" s="43"/>
       <c r="E89" s="43" t="s">
+        <v>383</v>
+      </c>
+      <c r="F89" s="51" t="s">
         <v>384</v>
       </c>
-      <c r="F89" s="51" t="s">
+      <c r="G89" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H89" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I89" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J89" s="50" t="s">
         <v>385</v>
       </c>
-      <c r="G89" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H89" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I89" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J89" s="50" t="s">
-        <v>386</v>
-      </c>
       <c r="K89" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6614,29 +6614,29 @@
         <v>2</v>
       </c>
       <c r="C90" s="43" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D90" s="43"/>
       <c r="E90" s="43" t="s">
+        <v>387</v>
+      </c>
+      <c r="F90" s="44" t="s">
         <v>388</v>
       </c>
-      <c r="F90" s="44" t="s">
+      <c r="G90" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H90" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I90" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J90" s="51" t="s">
         <v>389</v>
       </c>
-      <c r="G90" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H90" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I90" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J90" s="51" t="s">
-        <v>390</v>
-      </c>
       <c r="K90" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -6647,29 +6647,29 @@
         <v>2</v>
       </c>
       <c r="C91" s="43" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D91" s="43"/>
       <c r="E91" s="43" t="s">
+        <v>391</v>
+      </c>
+      <c r="F91" s="44" t="s">
         <v>392</v>
       </c>
-      <c r="F91" s="44" t="s">
+      <c r="G91" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H91" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I91" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J91" s="50" t="s">
         <v>393</v>
       </c>
-      <c r="G91" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H91" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I91" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J91" s="50" t="s">
-        <v>394</v>
-      </c>
       <c r="K91" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="55.2" x14ac:dyDescent="0.3">
@@ -6680,29 +6680,29 @@
         <v>2</v>
       </c>
       <c r="C92" s="43" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D92" s="43"/>
       <c r="E92" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="F92" s="43" t="s">
         <v>396</v>
       </c>
-      <c r="F92" s="43" t="s">
+      <c r="G92" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H92" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I92" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J92" s="50" t="s">
         <v>397</v>
       </c>
-      <c r="G92" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H92" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I92" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J92" s="50" t="s">
-        <v>398</v>
-      </c>
       <c r="K92" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6713,29 +6713,29 @@
         <v>2</v>
       </c>
       <c r="C93" s="43" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D93" s="43"/>
       <c r="E93" s="43" t="s">
+        <v>399</v>
+      </c>
+      <c r="F93" s="44" t="s">
         <v>400</v>
       </c>
-      <c r="F93" s="44" t="s">
+      <c r="G93" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H93" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I93" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J93" s="43" t="s">
         <v>401</v>
       </c>
-      <c r="G93" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H93" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I93" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J93" s="43" t="s">
-        <v>402</v>
-      </c>
       <c r="K93" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
@@ -6746,29 +6746,29 @@
         <v>2</v>
       </c>
       <c r="C94" s="43" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D94" s="43"/>
       <c r="E94" s="43" t="s">
+        <v>403</v>
+      </c>
+      <c r="F94" s="44" t="s">
         <v>404</v>
       </c>
-      <c r="F94" s="44" t="s">
+      <c r="G94" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H94" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I94" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J94" s="50" t="s">
         <v>405</v>
       </c>
-      <c r="G94" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H94" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I94" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J94" s="50" t="s">
-        <v>406</v>
-      </c>
       <c r="K94" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6779,29 +6779,29 @@
         <v>2</v>
       </c>
       <c r="C95" s="43" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D95" s="43"/>
       <c r="E95" s="43" t="s">
+        <v>407</v>
+      </c>
+      <c r="F95" s="44" t="s">
         <v>408</v>
       </c>
-      <c r="F95" s="44" t="s">
+      <c r="G95" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H95" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I95" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J95" s="51" t="s">
         <v>409</v>
       </c>
-      <c r="G95" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H95" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I95" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J95" s="51" t="s">
-        <v>410</v>
-      </c>
       <c r="K95" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="72" x14ac:dyDescent="0.3">
@@ -6812,29 +6812,29 @@
         <v>2</v>
       </c>
       <c r="C96" s="43" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D96" s="43"/>
       <c r="E96" s="43" t="s">
+        <v>411</v>
+      </c>
+      <c r="F96" s="44" t="s">
         <v>412</v>
       </c>
-      <c r="F96" s="44" t="s">
+      <c r="G96" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H96" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I96" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J96" s="50" t="s">
         <v>413</v>
       </c>
-      <c r="G96" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H96" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I96" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J96" s="50" t="s">
-        <v>414</v>
-      </c>
       <c r="K96" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="96.6" x14ac:dyDescent="0.3">
@@ -6845,29 +6845,29 @@
         <v>2</v>
       </c>
       <c r="C97" s="43" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D97" s="43"/>
       <c r="E97" s="43" t="s">
+        <v>415</v>
+      </c>
+      <c r="F97" s="43" t="s">
         <v>416</v>
       </c>
-      <c r="F97" s="43" t="s">
+      <c r="G97" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H97" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I97" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J97" s="51" t="s">
         <v>417</v>
       </c>
-      <c r="G97" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H97" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I97" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J97" s="51" t="s">
-        <v>418</v>
-      </c>
       <c r="K97" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -6878,29 +6878,29 @@
         <v>2</v>
       </c>
       <c r="C98" s="43" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D98" s="43"/>
       <c r="E98" s="44" t="s">
+        <v>419</v>
+      </c>
+      <c r="F98" s="44" t="s">
         <v>420</v>
       </c>
-      <c r="F98" s="44" t="s">
+      <c r="G98" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="H98" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I98" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J98" s="50" t="s">
         <v>421</v>
       </c>
-      <c r="G98" s="43" t="s">
-        <v>361</v>
-      </c>
-      <c r="H98" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I98" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J98" s="50" t="s">
-        <v>422</v>
-      </c>
       <c r="K98" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.3">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="D99" s="43"/>
       <c r="E99" s="44" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F99" s="44"/>
       <c r="G99" s="43"/>
@@ -6930,29 +6930,29 @@
         <v>2</v>
       </c>
       <c r="C100" s="43" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D100" s="43"/>
       <c r="E100" s="43" t="s">
+        <v>424</v>
+      </c>
+      <c r="F100" s="44" t="s">
         <v>425</v>
       </c>
-      <c r="F100" s="44" t="s">
+      <c r="G100" s="43" t="s">
         <v>426</v>
       </c>
-      <c r="G100" s="43" t="s">
+      <c r="H100" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I100" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J100" s="44" t="s">
         <v>427</v>
       </c>
-      <c r="H100" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I100" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J100" s="44" t="s">
-        <v>428</v>
-      </c>
       <c r="K100" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -6963,29 +6963,29 @@
         <v>2</v>
       </c>
       <c r="C101" s="43" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D101" s="43"/>
       <c r="E101" s="43" t="s">
+        <v>429</v>
+      </c>
+      <c r="F101" s="44" t="s">
         <v>430</v>
       </c>
-      <c r="F101" s="44" t="s">
+      <c r="G101" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H101" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I101" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J101" s="53" t="s">
         <v>431</v>
       </c>
-      <c r="G101" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H101" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I101" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J101" s="53" t="s">
-        <v>432</v>
-      </c>
       <c r="K101" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -6996,29 +6996,29 @@
         <v>2</v>
       </c>
       <c r="C102" s="43" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D102" s="43"/>
       <c r="E102" s="43" t="s">
+        <v>433</v>
+      </c>
+      <c r="F102" s="44" t="s">
         <v>434</v>
       </c>
-      <c r="F102" s="44" t="s">
+      <c r="G102" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H102" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I102" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J102" s="50" t="s">
         <v>435</v>
       </c>
-      <c r="G102" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H102" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I102" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J102" s="50" t="s">
-        <v>436</v>
-      </c>
       <c r="K102" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="138" x14ac:dyDescent="0.3">
@@ -7029,29 +7029,29 @@
         <v>2</v>
       </c>
       <c r="C103" s="43" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D103" s="43"/>
       <c r="E103" s="43" t="s">
+        <v>437</v>
+      </c>
+      <c r="F103" s="44" t="s">
         <v>438</v>
       </c>
-      <c r="F103" s="44" t="s">
+      <c r="G103" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H103" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I103" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J103" s="51" t="s">
         <v>439</v>
       </c>
-      <c r="G103" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H103" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I103" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J103" s="51" t="s">
-        <v>440</v>
-      </c>
       <c r="K103" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="69" x14ac:dyDescent="0.3">
@@ -7062,29 +7062,29 @@
         <v>2</v>
       </c>
       <c r="C104" s="43" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D104" s="43"/>
       <c r="E104" s="43" t="s">
+        <v>441</v>
+      </c>
+      <c r="F104" s="43" t="s">
         <v>442</v>
       </c>
-      <c r="F104" s="43" t="s">
+      <c r="G104" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H104" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I104" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J104" s="51" t="s">
         <v>443</v>
       </c>
-      <c r="G104" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H104" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I104" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J104" s="51" t="s">
-        <v>444</v>
-      </c>
       <c r="K104" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
@@ -7095,29 +7095,29 @@
         <v>2</v>
       </c>
       <c r="C105" s="43" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D105" s="43"/>
       <c r="E105" s="43" t="s">
+        <v>445</v>
+      </c>
+      <c r="F105" s="54" t="s">
         <v>446</v>
       </c>
-      <c r="F105" s="54" t="s">
+      <c r="G105" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H105" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I105" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J105" s="50" t="s">
         <v>447</v>
       </c>
-      <c r="G105" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H105" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I105" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J105" s="50" t="s">
-        <v>448</v>
-      </c>
       <c r="K105" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -7128,29 +7128,29 @@
         <v>2</v>
       </c>
       <c r="C106" s="43" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D106" s="43"/>
       <c r="E106" s="43" t="s">
+        <v>449</v>
+      </c>
+      <c r="F106" s="43" t="s">
         <v>450</v>
       </c>
-      <c r="F106" s="43" t="s">
+      <c r="G106" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H106" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I106" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J106" s="51" t="s">
         <v>451</v>
       </c>
-      <c r="G106" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H106" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I106" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J106" s="51" t="s">
-        <v>452</v>
-      </c>
       <c r="K106" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="110.4" x14ac:dyDescent="0.3">
@@ -7161,29 +7161,29 @@
         <v>2</v>
       </c>
       <c r="C107" s="43" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D107" s="43"/>
       <c r="E107" s="43" t="s">
+        <v>453</v>
+      </c>
+      <c r="F107" s="54" t="s">
         <v>454</v>
       </c>
-      <c r="F107" s="54" t="s">
+      <c r="G107" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H107" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I107" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J107" s="51" t="s">
         <v>455</v>
       </c>
-      <c r="G107" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H107" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I107" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J107" s="51" t="s">
-        <v>456</v>
-      </c>
       <c r="K107" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
@@ -7194,29 +7194,29 @@
         <v>2</v>
       </c>
       <c r="C108" s="43" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D108" s="43"/>
       <c r="E108" s="43" t="s">
+        <v>457</v>
+      </c>
+      <c r="F108" s="43" t="s">
         <v>458</v>
       </c>
-      <c r="F108" s="43" t="s">
+      <c r="G108" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H108" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I108" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J108" s="43" t="s">
         <v>459</v>
       </c>
-      <c r="G108" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H108" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I108" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J108" s="43" t="s">
-        <v>460</v>
-      </c>
       <c r="K108" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -7227,29 +7227,29 @@
         <v>2</v>
       </c>
       <c r="C109" s="43" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D109" s="43"/>
       <c r="E109" s="44" t="s">
+        <v>461</v>
+      </c>
+      <c r="F109" s="44" t="s">
         <v>462</v>
       </c>
-      <c r="F109" s="44" t="s">
+      <c r="G109" s="44" t="s">
+        <v>426</v>
+      </c>
+      <c r="H109" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I109" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J109" s="44" t="s">
         <v>463</v>
       </c>
-      <c r="G109" s="44" t="s">
-        <v>427</v>
-      </c>
-      <c r="H109" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I109" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J109" s="44" t="s">
-        <v>464</v>
-      </c>
       <c r="K109" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
@@ -7260,29 +7260,29 @@
         <v>2</v>
       </c>
       <c r="C110" s="43" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D110" s="43"/>
       <c r="E110" s="43" t="s">
+        <v>465</v>
+      </c>
+      <c r="F110" s="43" t="s">
         <v>466</v>
       </c>
-      <c r="F110" s="43" t="s">
+      <c r="G110" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H110" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I110" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J110" s="50" t="s">
         <v>467</v>
       </c>
-      <c r="G110" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H110" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I110" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J110" s="50" t="s">
-        <v>468</v>
-      </c>
       <c r="K110" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
@@ -7293,29 +7293,29 @@
         <v>2</v>
       </c>
       <c r="C111" s="43" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D111" s="43"/>
       <c r="E111" s="43" t="s">
+        <v>469</v>
+      </c>
+      <c r="F111" s="44" t="s">
         <v>470</v>
       </c>
-      <c r="F111" s="44" t="s">
+      <c r="G111" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H111" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I111" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J111" s="50" t="s">
         <v>471</v>
       </c>
-      <c r="G111" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H111" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I111" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J111" s="50" t="s">
-        <v>472</v>
-      </c>
       <c r="K111" s="55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
@@ -7326,29 +7326,29 @@
         <v>2</v>
       </c>
       <c r="C112" s="43" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D112" s="43"/>
       <c r="E112" s="43" t="s">
+        <v>473</v>
+      </c>
+      <c r="F112" s="44" t="s">
         <v>474</v>
       </c>
-      <c r="F112" s="44" t="s">
+      <c r="G112" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H112" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I112" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J112" s="51" t="s">
         <v>475</v>
       </c>
-      <c r="G112" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H112" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I112" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J112" s="51" t="s">
-        <v>476</v>
-      </c>
       <c r="K112" s="55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="72" x14ac:dyDescent="0.3">
@@ -7359,29 +7359,29 @@
         <v>2</v>
       </c>
       <c r="C113" s="43" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D113" s="43"/>
       <c r="E113" s="43" t="s">
+        <v>477</v>
+      </c>
+      <c r="F113" s="44" t="s">
         <v>478</v>
       </c>
-      <c r="F113" s="44" t="s">
+      <c r="G113" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="H113" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="I113" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="J113" s="50" t="s">
         <v>479</v>
       </c>
-      <c r="G113" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="H113" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="I113" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="J113" s="50" t="s">
-        <v>480</v>
-      </c>
       <c r="K113" s="56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -7453,24 +7453,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -7537,13 +7537,13 @@
     </row>
     <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>